<commit_message>
Pool：池数量 Procedure：注册数量、当前状态、状态持续时间 UI：管理中的 UI Window 数量 Entity：实体和实体组数量 Config：已加载配置表数量 Localization：当前语言、已加载及支持语言数量 Resource：已加载、加载中的资源数量 Scene：当前场景、已加载及加载中场景数量 Network：通道数、默认通道及连接地址 Audio：缓存数、当前 BGM、播放状态、音量 FSM、Event、Timer、WebRequest、Debugger、Base：各自核心运行数据 新增 GameEntry.Restart() 统一重启入口：[GameEntry.cs (line 337)](E:/ProJect/Unity/UnityRFramework/Assets/UnityRFramework/Scripts/Runtime/GameEntry.cs:337) 重启前同步关闭全部模块、停止协程并解除回调：[BaseComponent.cs (line 224)](E:/ProJect/Unity/UnityRFramework/Assets/UnityRFramework/Scripts/Runtime/Base/BaseComponent.cs:224) 清理 GameEntry 中指向旧组件的静态缓存，避免重启后访问已释放模块：[GameEntry.cs (line 354)](E:/ProJect/Unity/UnityRFramework/Assets/UnityRFramework/Scripts/Runtime/GameEntry.cs:354) 大厅顶栏新增 ↻ 重启按钮：[DemoTopBar.cs (line 114)](E:/ProJect/Unity/UnityRFramework/Assets/UnityRFramework/Samples/Demo/Scripts/Hall/DemoTopBar.cs:114) Demo 两份 README 均已补充软重启验收说明：[README.md (line 60)](E:/ProJect/Unity/UnityRFramework/Assets/UnityRFramework/Samples/Demo/README.md:60)
</commit_message>
<xml_diff>
--- a/Samples~/Demo/ConfigSource/Localization/en.xlsx
+++ b/Samples~/Demo/ConfigSource/Localization/en.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Localization" sheetId="1" r:id="R4a5d3631c54144a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Localization" sheetId="1" r:id="Rc82ad12133e9492e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -143,7 +143,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="en_Table" displayName="en_Table" ref="A1:B72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="en_Table" displayName="en_Table" ref="A1:B74" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Key"/>
     <x:tableColumn id="2" name="Value"/>
@@ -948,10 +948,26 @@
         <x:v>English</x:v>
       </x:c>
     </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>UI_Restart</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>Restart</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>UI_Quit</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>Quit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebe04cdeb11d4c96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ecaa44f3cf549e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>